<commit_message>
Replace old 30-day plan with the new advanced topic list
The Markdown plan is now generated from make_sheet.py, so it matches the sheet.
Removes the basic topics (background removal, object removal, PDF tools).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013EjpVZtyDnYNbzPcyvRsPV
</commit_message>
<xml_diff>
--- a/content/subscription-band-karo-30-days.xlsx
+++ b/content/subscription-band-karo-30-days.xlsx
@@ -1586,7 +1586,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Koi bhi article ya PDF, aur do AI hosts uspe podcast karenge.</t>
+          <t>Koi bhi article, notes ya YouTube video, aur do AI hosts uspe podcast karenge.</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
@@ -1611,10 +1611,10 @@
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>Koi bhi article ya PDF, aur do AI hosts uspe podcast karenge.
+          <t>Koi bhi article, notes ya YouTube video, aur do AI hosts uspe podcast karenge.
 Subscription Band Karo, Day 16.
 NotebookLM ka podcast feature sabko pasand aaya. Podcastfy uska open-source version hai.
-Article, PDF, ya YouTube video do, aur ye do logon ki natural baatcheet waala podcast bana deta hai. Padhai karte hue suno, ya apne content ko audio mein badlo.
+Article, notes, ya YouTube video do, aur ye do logon ki natural baatcheet waala podcast bana deta hai. Padhai karte hue suno, ya apne content ko audio mein badlo.
 Aur kyunki ye open source hai, tum awaaz, style aur language khud choose kar sakte ho.
 AI model aur voice ke liye API key ya local model lagta hai.
 Link chahiye? Comment karo PODCAST. Kal Day 17 mein, apna ChatGPT, bina internet. Bye!</t>

</xml_diff>

<commit_message>
Day 1 script: add series line and Day 2 teaser
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013EjpVZtyDnYNbzPcyvRsPV
</commit_message>
<xml_diff>
--- a/content/subscription-band-karo-30-days.xlsx
+++ b/content/subscription-band-karo-30-days.xlsx
@@ -589,7 +589,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="360" customHeight="1">
+    <row r="2" ht="405" customHeight="1">
       <c r="A2" s="2" t="n">
         <v>1</v>
       </c>
@@ -631,12 +631,13 @@
       <c r="I2" s="4" t="inlineStr">
         <is>
           <t>Bhai, tum abhi bhi in AI tools ke liye paise de rahe ho? Inke FREE versions exist karte hain! Aur number one dekh ke tum shock ho jaoge.
+Subscription Band Karo, Day 1.
 Number 5. Transcription ke paise? Buzz kisi bhi video ke subtitles bana deta hai, wo bhi bina internet ke. Tumhara data laptop se bahar hi nahi jaata.
 Number 4. Grammarly Premium? Chhodo! LanguageTool pachchees se zyada languages mein tumhari grammar fix karta hai, aur ye open source hai.
 Number 3. Photo blurry hai? Upscayl mein daalo, kuch seconds mein ekdum HD. GitHub pe pachaas hazaar se zyada logon ne isse star kiya hai.
 Number 2. Midjourney har mahine paise kaat-ta hai. ComfyUI tumhare apne PC pe AI images banata hai. Na monthly bill, na koi tension.
 Aur number 1. ElevenLabs ka bilkul free, open-source alternative! VoiceStudio voice clone karta hai, videos dub karta hai, audiobooks banata hai, sab tumhare computer pe.
-Saare links chahiye? Follow karo aur comment karo TOOLS. Main seedha DM kar dunga. Bye!</t>
+Saare links chahiye? Follow karo aur comment karo TOOLS. Main seedha DM kar dunga. Kal Day 2 mein, ek free AI engineer jo tumhare liye poora app likhega. Bye!</t>
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr">
@@ -646,12 +647,12 @@
       </c>
       <c r="K2" s="4" t="inlineStr">
         <is>
-          <t>Already built (5-paid-ai-tools example).</t>
+          <t>Already built (5-paid-ai-tools example). Script now adds the series line and the Day 2 teaser: re-record the voiceover if you want them spoken.</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Recorded</t>
+          <t>Script ready</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Content sheet: single tab with how-to notes under the table
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013EjpVZtyDnYNbzPcyvRsPV
</commit_message>
<xml_diff>
--- a/content/subscription-band-karo-30-days.xlsx
+++ b/content/subscription-band-karo-30-days.xlsx
@@ -8,7 +8,6 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="30-Day Plan" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to use" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'30-Day Plan'!$A$1:$L$31</definedName>
@@ -20,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -42,20 +41,6 @@
       <name val="Arial"/>
       <b val="1"/>
       <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <sz val="16"/>
     </font>
   </fonts>
   <fills count="5">
@@ -107,7 +92,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -136,13 +121,8 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -510,7 +490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L31"/>
+  <dimension ref="A1:L37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2534,8 +2514,80 @@
         </is>
       </c>
     </row>
+    <row r="33" ht="18" customHeight="1">
+      <c r="A33" s="10" t="inlineStr">
+        <is>
+          <t>HOW TO USE</t>
+        </is>
+      </c>
+      <c r="C33" s="11" t="inlineStr">
+        <is>
+          <t>Edit only column L (Status) as you go: To do · Script ready · Voice recorded · Video built · Posted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="18" customHeight="1">
+      <c r="A34" s="10" t="inlineStr">
+        <is>
+          <t>Workflow</t>
+        </is>
+      </c>
+      <c r="C34" s="11" t="inlineStr">
+        <is>
+          <t>Paste the Voice Script into your voice tool → send me the audio → the freestack-video skill builds the reel → post with the Post Title.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="18" customHeight="1">
+      <c r="A35" s="10" t="inlineStr">
+        <is>
+          <t>Caption</t>
+        </is>
+      </c>
+      <c r="C35" s="11" t="inlineStr">
+        <is>
+          <t>Hook line · one line on the tool + its catch · Comment "&lt;KEYWORD&gt;" for the link · Follow @freestack.ai · 5–8 hashtags</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="18" customHeight="1">
+      <c r="A36" s="10" t="inlineStr">
+        <is>
+          <t>ManyChat</t>
+        </is>
+      </c>
+      <c r="C36" s="11" t="inlineStr">
+        <is>
+          <t>One keyword automation per day (column H) that DMs that day's links.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="18" customHeight="1">
+      <c r="A37" s="10" t="inlineStr">
+        <is>
+          <t>Accuracy</t>
+        </is>
+      </c>
+      <c r="C37" s="11" t="inlineStr">
+        <is>
+          <t>Repos checked on GitHub on 15 Oct 2026. Star counts are not spoken; the video shows the live count.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:L31"/>
+  <mergeCells count="10">
+    <mergeCell ref="C36:I36"/>
+    <mergeCell ref="C37:I37"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="C35:I35"/>
+    <mergeCell ref="C34:I34"/>
+    <mergeCell ref="A37:B37"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="C33:I33"/>
+    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="A35:B35"/>
+  </mergeCells>
   <dataValidations count="1">
     <dataValidation sqref="L2:L31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"To do,Script ready,Voice recorded,Video built,Posted"</formula1>
@@ -2543,118 +2595,4 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="110" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="10" t="inlineStr">
-        <is>
-          <t>Subscription Band Karo: 30-Day Series</t>
-        </is>
-      </c>
-      <c r="B1" s="11" t="inlineStr"/>
-    </row>
-    <row r="2">
-      <c r="A2" s="11" t="inlineStr"/>
-      <c r="B2" s="12" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="11" t="inlineStr">
-        <is>
-          <t>Edit only</t>
-        </is>
-      </c>
-      <c r="B3" s="12" t="inlineStr">
-        <is>
-          <t>Column L (Status) on the 30-Day Plan tab: pick from the dropdown as you go.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="11" t="inlineStr">
-        <is>
-          <t>Workflow</t>
-        </is>
-      </c>
-      <c r="B4" s="12" t="inlineStr">
-        <is>
-          <t>1) Paste the Voice Script into your voice tool → 2) send me the audio → 3) the freestack-video skill builds the reel → 4) post with the Post Title + caption.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="11" t="inlineStr">
-        <is>
-          <t>Post title</t>
-        </is>
-      </c>
-      <c r="B5" s="12" t="inlineStr">
-        <is>
-          <t>Day (X/30) Subscription Band Karo: &lt;topic&gt;</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="11" t="inlineStr">
-        <is>
-          <t>Caption</t>
-        </is>
-      </c>
-      <c r="B6" s="12" t="inlineStr">
-        <is>
-          <t>Hook line · one line on the tool + its catch · Comment "&lt;KEYWORD&gt;" for the link · Follow @freestack.ai · 5–8 hashtags</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="11" t="inlineStr">
-        <is>
-          <t>ManyChat</t>
-        </is>
-      </c>
-      <c r="B7" s="12" t="inlineStr">
-        <is>
-          <t>Create one keyword automation per day (column H) that DMs that day's links.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="11" t="inlineStr">
-        <is>
-          <t>Accuracy</t>
-        </is>
-      </c>
-      <c r="B8" s="12" t="inlineStr">
-        <is>
-          <t>Repos were checked on GitHub on 15 Oct 2026. Star counts are not spoken; the video shows the live count.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="11" t="inlineStr">
-        <is>
-          <t>Status values</t>
-        </is>
-      </c>
-      <c r="B9" s="12" t="inlineStr">
-        <is>
-          <t>To do · Script ready · Voice recorded · Video built · Posted</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>